<commit_message>
General files structure refactoring
</commit_message>
<xml_diff>
--- a/modules/on_off_module_x1/PCB/Outputs/BOM/on_off_module_x1.xlsx
+++ b/modules/on_off_module_x1/PCB/Outputs/BOM/on_off_module_x1.xlsx
@@ -446,12 +446,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -585,12 +585,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>220nF</t>
+          <t>47nF - 350V</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>CAP_THT_CERAMIC_X2_13x6x12</t>
+          <t>CAP_THT_CERAMIC_X2_13x5x11_P10</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -600,17 +600,17 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>LED</t>
+          <t>100nF - 6,3V</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>LED_SMD_0603</t>
+          <t>CAP_SMD_CERAMIC_0603</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -620,17 +620,17 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>DIODE_SMD_SOD323F</t>
+          <t>LED_SMD_0603</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
@@ -640,37 +640,37 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>J1, J2, J3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Screw_Terminal_01x02</t>
+          <t>S1A</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>CONN_TERMINAL-BLOCK_2P_P5.08</t>
+          <t>DIODE_SMD_SMA</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Conn_01x06_Socket</t>
+          <t>0,25A - 250V</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>CONN_SOCKET-HEADER_1x06_V</t>
+          <t>FUSEHOLDER_THT_5x20_CLIP</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
@@ -680,17 +680,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Conn_01x03_Socket</t>
+          <t>CONN_TERMINAL-BLOCK_5P_P5.08</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>CONN_PIN-HEADER_1x03_V</t>
+          <t>CONN_TERMINAL-BLOCK_5P_P5.08</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
@@ -700,17 +700,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>12V 5A</t>
+          <t>Conn_01x06_Socket</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>RELAY_SPDT_FINDER_36.11</t>
+          <t>CONN_SOCKET-HEADER_1x06_V</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
@@ -720,17 +720,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>PS1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>HLK-PM12 - 3W</t>
+          <t>Conn_01x03_Socket</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>HILINK_HLK-PMxx</t>
+          <t>CONN_PIN-HEADER_1x03_V</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -740,17 +740,17 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>2N7002H</t>
+          <t>12V 5A</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>RELAY_SPDT_FINDER_36.11</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -760,17 +760,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>600R</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>RES_SMD_1206</t>
+          <t>BEAD_SMD_1206</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
@@ -780,17 +780,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>PS1</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>390 - 5% - 1/10W</t>
+          <t>HLK-PM12 - 3W</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>RES_SMD_0603</t>
+          <t>HILINK_HLK-PMxx</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
@@ -800,37 +800,37 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>R1, R2, R3, R6</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>10k - 5% - 1/10W</t>
+          <t>2N7002H</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>RES_SMD_0603</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>R4, R7</t>
+          <t>R10, R11</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>2.2k - 5% - 1/10W</t>
+          <t>33k - 5% - 1/4W</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>RES_SMD_0603</t>
+          <t>RES_SMD_1206</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
@@ -840,37 +840,37 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R1, R2, R3, R6, R12</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>10k - 5% - 1/10W</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>LDR_5_V</t>
+          <t>RES_SMD_0603</t>
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>2k2 - 5% - 1/10W</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>RES_SMD_1206</t>
+          <t>RES_SMD_0603</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
@@ -880,17 +880,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SW_SPDT</t>
+          <t>390R - 5% - 1/10W</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>SW_TOGGLE_DPDT_THT_7x7</t>
+          <t>RES_SMD_0603</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
@@ -900,17 +900,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>AMS1117-3.3 - 3.3W</t>
+          <t>33k - 5% - 1/10W</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>SOT-223-3_TAB2</t>
+          <t>RES_SMD_0603</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
@@ -920,17 +920,17 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>ESP-12E</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>MOD_ESP-12E</t>
+          <t>LDR_5_V</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
@@ -940,17 +940,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>PC817</t>
+          <t>470k - 5% - 1/4W</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>SMDIP-4_7.62</t>
+          <t>RES_SMD_1206</t>
         </is>
       </c>
       <c r="D25" s="4" t="n">
@@ -960,20 +960,80 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>AMS1117-3.3 - 3.3W</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>SOT-223-3_TAB2</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>ESP-12E</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>MOD_ESP-12E</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>PC817</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>SMDIP-4_7.62</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
           <t>U4</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>H11AA1</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>SMDIP-6_7.62</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D29" s="4" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>